<commit_message>
Arregle algunas cosas, solo agregue para modificar las zonas y loa biggies pero es un ruteo donde descargar un excel y al examinar un archivo el sistema automaticamente te hace un ruteo, cada empleado por su zona
</commit_message>
<xml_diff>
--- a/Desktop/biggie-ruteo-paraguay/sample_data/plantilla_rutas_biggie.xlsx
+++ b/Desktop/biggie-ruteo-paraguay/sample_data/plantilla_rutas_biggie.xlsx
@@ -397,443 +397,137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:C11"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="42.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ID Sucursal</v>
+        <v>Empleado</v>
       </c>
       <c r="B1" t="str">
-        <v>Nombre Sucursal</v>
+        <v>Sucursal</v>
       </c>
       <c r="C1" t="str">
-        <v>Direccion</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Ciudad</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Zona</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Latitud</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Longitud</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Nro Pedido</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Cajas/Bultos</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Prioridad</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Telefono Contacto</v>
-      </c>
-      <c r="L1" t="str">
         <v>Notas</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BIG-VM-01</v>
+        <v>Carlos Gómez</v>
       </c>
       <c r="B2" t="str">
         <v>Biggie Villa Morra</v>
       </c>
       <c r="C2" t="str">
-        <v>Avda. Mariscal López c/ Senador Long</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Asunción</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Villa Morra</v>
-      </c>
-      <c r="F2">
-        <v>-25.2971</v>
-      </c>
-      <c r="G2">
-        <v>-57.5866</v>
-      </c>
-      <c r="H2" t="str">
-        <v>PED-2026-081</v>
-      </c>
-      <c r="I2">
-        <v>15</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Alta</v>
-      </c>
-      <c r="K2" t="str">
-        <v>0981 200001</v>
-      </c>
-      <c r="L2" t="str">
         <v>Entregar por portón lateral</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BIG-ASU-01</v>
+        <v>Carlos Gómez</v>
       </c>
       <c r="B3" t="str">
         <v>Biggie Palma</v>
       </c>
       <c r="C3" t="str">
-        <v>Calle Palma e/ 14 de Mayo y 15 de Agosto</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Asunción</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Palma Centro</v>
-      </c>
-      <c r="F3">
-        <v>-25.2833</v>
-      </c>
-      <c r="G3">
-        <v>-57.6331</v>
-      </c>
-      <c r="H3" t="str">
-        <v>PED-2026-082</v>
-      </c>
-      <c r="I3">
-        <v>12</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K3" t="str">
-        <v>0981 100001</v>
-      </c>
-      <c r="L3" t="str">
         <v>Recepción abierta 24hs</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BIG-LUQ-01</v>
+        <v>María López</v>
       </c>
       <c r="B4" t="str">
         <v>Biggie Luque Centro</v>
       </c>
       <c r="C4" t="str">
-        <v>Gral. Aquino c/ Rosario</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Luque</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Luque Centro</v>
-      </c>
-      <c r="F4">
-        <v>-25.2668</v>
-      </c>
-      <c r="G4">
-        <v>-57.4962</v>
-      </c>
-      <c r="H4" t="str">
-        <v>PED-2026-086</v>
-      </c>
-      <c r="I4">
-        <v>14</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K4" t="str">
-        <v>0981 300001</v>
-      </c>
-      <c r="L4" t="str">
         <v>Frente a plaza principal</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BIG-MRA-01</v>
+        <v>María López</v>
       </c>
       <c r="B5" t="str">
         <v>Biggie Mariano Roque Alonso</v>
       </c>
       <c r="C5" t="str">
-        <v>Ruta Transchaco c/ Bernardino Caballero</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Mariano Roque Alonso</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Mariano Roque Alonso Transchaco</v>
-      </c>
-      <c r="F5">
-        <v>-25.2289</v>
-      </c>
-      <c r="G5">
-        <v>-57.5342</v>
-      </c>
-      <c r="H5" t="str">
-        <v>PED-2026-088</v>
-      </c>
-      <c r="I5">
-        <v>22</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Alta</v>
-      </c>
-      <c r="K5" t="str">
-        <v>0981 300003</v>
-      </c>
-      <c r="L5" t="str">
         <v>Descarga en bahía de camiones</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BIG-SL-01</v>
+        <v>Juan Pérez</v>
       </c>
       <c r="B6" t="str">
         <v>Biggie San Lorenzo Centro</v>
       </c>
       <c r="C6" t="str">
-        <v>Julia Miranda Cueto c/ Sgto. Silva</v>
-      </c>
-      <c r="D6" t="str">
-        <v>San Lorenzo</v>
-      </c>
-      <c r="E6" t="str">
-        <v>San Lorenzo Centro</v>
-      </c>
-      <c r="F6">
-        <v>-25.3212</v>
-      </c>
-      <c r="G6">
-        <v>-57.4974</v>
-      </c>
-      <c r="H6" t="str">
-        <v>PED-2026-089</v>
-      </c>
-      <c r="I6">
-        <v>16</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K6" t="str">
-        <v>0981 400001</v>
-      </c>
-      <c r="L6" t="str">
         <v>Zona comercial centro</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BIG-CAP-01</v>
+        <v>Juan Pérez</v>
       </c>
       <c r="B7" t="str">
         <v>Biggie Capiatá Km 16</v>
       </c>
       <c r="C7" t="str">
-        <v>Ruta PY02 Km 16.5 c/ Aratiri</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Capiatá</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Capiatá Km 16 Aratiri</v>
-      </c>
-      <c r="F7">
-        <v>-25.3585</v>
-      </c>
-      <c r="G7">
-        <v>-57.4372</v>
-      </c>
-      <c r="H7" t="str">
-        <v>PED-2026-094</v>
-      </c>
-      <c r="I7">
-        <v>18</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K7" t="str">
-        <v>0981 400004</v>
-      </c>
-      <c r="L7" t="str">
         <v>Entrada por colectora</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BIG-FDM-01</v>
+        <v>Ana Martínez</v>
       </c>
       <c r="B8" t="str">
         <v>Biggie Fernando Norte</v>
       </c>
       <c r="C8" t="str">
-        <v>Avda. Mcal. López c/ Insaurralde</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Fernando de la Mora</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Fernando de la Mora Norte</v>
-      </c>
-      <c r="F8">
-        <v>-25.3074</v>
-      </c>
-      <c r="G8">
-        <v>-57.5332</v>
-      </c>
-      <c r="H8" t="str">
-        <v>PED-2026-091</v>
-      </c>
-      <c r="I8">
-        <v>11</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K8" t="str">
-        <v>0981 500001</v>
-      </c>
-      <c r="L8" t="str">
         <v>Lado norte</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BIG-LAM-01</v>
+        <v>Ana Martínez</v>
       </c>
       <c r="B9" t="str">
         <v>Biggie Lambaré</v>
       </c>
       <c r="C9" t="str">
-        <v>Avda. Cacique Lambaré c/ Río Apa</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Lambaré</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Lambaré Cacique</v>
-      </c>
-      <c r="F9">
-        <v>-25.3389</v>
-      </c>
-      <c r="G9">
-        <v>-57.6184</v>
-      </c>
-      <c r="H9" t="str">
-        <v>PED-2026-092</v>
-      </c>
-      <c r="I9">
-        <v>15</v>
-      </c>
-      <c r="J9" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K9" t="str">
-        <v>0981 600001</v>
-      </c>
-      <c r="L9" t="str">
         <v>Estacionamiento amplio</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>BIG-VEL-01</v>
+        <v>Pedro Ramírez</v>
       </c>
       <c r="B10" t="str">
         <v>Biggie Villa Elisa</v>
       </c>
       <c r="C10" t="str">
-        <v>Avda. Von Poleski c/ Colombia</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Villa Elisa</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Villa Elisa Centro</v>
-      </c>
-      <c r="F10">
-        <v>-25.3697</v>
-      </c>
-      <c r="G10">
-        <v>-57.5839</v>
-      </c>
-      <c r="H10" t="str">
-        <v>PED-2026-095</v>
-      </c>
-      <c r="I10">
-        <v>13</v>
-      </c>
-      <c r="J10" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K10" t="str">
-        <v>0981 600003</v>
-      </c>
-      <c r="L10" t="str">
         <v>Sobre avenida principal</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>BIG-NEM-01</v>
+        <v>Pedro Ramírez</v>
       </c>
       <c r="B11" t="str">
         <v>Biggie Ñemby</v>
       </c>
       <c r="C11" t="str">
-        <v>Avda. Acceso Sur c/ Pratt Gill</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Ñemby</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Ñemby Acceso Sur</v>
-      </c>
-      <c r="F11">
-        <v>-25.4014</v>
-      </c>
-      <c r="G11">
-        <v>-57.5753</v>
-      </c>
-      <c r="H11" t="str">
-        <v>PED-2026-096</v>
-      </c>
-      <c r="I11">
-        <v>20</v>
-      </c>
-      <c r="J11" t="str">
-        <v>Alta</v>
-      </c>
-      <c r="K11" t="str">
-        <v>0981 600004</v>
-      </c>
-      <c r="L11" t="str">
         <v>Descarga en patio trasero</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>